<commit_message>
Negative case for Search employee commit
</commit_message>
<xml_diff>
--- a/PROJECT_OHRM/test_data/DirectoryData.xlsx
+++ b/PROJECT_OHRM/test_data/DirectoryData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e8f8df283bc7727/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e8f8df283bc7727/Desktop/Testing modules/OrangeHRM/OHRM_Project/PROJECT_OHRM/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{882AF23D-0A72-4ADC-8220-62711CABB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{187D950D-07E6-4206-A6B5-8CE32AC34AD8}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{882AF23D-0A72-4ADC-8220-62711CABB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D75EEE1-8382-486D-9804-25B8592C68B0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BA2B306-E5DF-4422-BA37-E21C05DD95BD}"/>
   </bookViews>
@@ -34,12 +34,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>EmployeeName</t>
   </si>
   <si>
     <t>Ranga</t>
+  </si>
+  <si>
+    <t>Linda</t>
   </si>
 </sst>
 </file>
@@ -411,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25209873-7B8E-481A-A82B-2CD633758F84}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -424,6 +427,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Modified test data file in the directory
</commit_message>
<xml_diff>
--- a/PROJECT_OHRM/test_data/DirectoryData.xlsx
+++ b/PROJECT_OHRM/test_data/DirectoryData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e8f8df283bc7727/Desktop/Testing modules/OrangeHRM/OHRM_Project/PROJECT_OHRM/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{882AF23D-0A72-4ADC-8220-62711CABB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D75EEE1-8382-486D-9804-25B8592C68B0}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{882AF23D-0A72-4ADC-8220-62711CABB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12562672-C097-4113-B1A2-D500E5C0C5AE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BA2B306-E5DF-4422-BA37-E21C05DD95BD}"/>
   </bookViews>
@@ -39,10 +39,10 @@
     <t>EmployeeName</t>
   </si>
   <si>
-    <t>Ranga</t>
+    <t>Linda</t>
   </si>
   <si>
-    <t>Linda</t>
+    <t>Admin</t>
   </si>
 </sst>
 </file>
@@ -95,6 +95,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -424,12 +428,12 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Searching employee by the location code commit
</commit_message>
<xml_diff>
--- a/PROJECT_OHRM/test_data/DirectoryData.xlsx
+++ b/PROJECT_OHRM/test_data/DirectoryData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e8f8df283bc7727/Desktop/Testing modules/OrangeHRM/OHRM_Project/PROJECT_OHRM/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{882AF23D-0A72-4ADC-8220-62711CABB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12562672-C097-4113-B1A2-D500E5C0C5AE}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{882AF23D-0A72-4ADC-8220-62711CABB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2039A9D8-0104-46B8-909C-60D6124B24C6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BA2B306-E5DF-4422-BA37-E21C05DD95BD}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <t>Linda</t>
   </si>
   <si>
-    <t>Admin</t>
+    <t>James</t>
   </si>
 </sst>
 </file>

</xml_diff>